<commit_message>
feat: add FastAPI web framework and pricing API endpoint
- Add FastAPI and uvicorn dependencies to support web API functionality
- Create new routers package with pricing endpoint for document processing
- Refactor parallel processing logic into utils.pipeline module
- Update VS Code import completions for FastAPI components

This enables the application to serve document processing and wage lookup functionality via HTTP API instead of just CLI batch processing.
</commit_message>
<xml_diff>
--- a/final_pricing.xlsx
+++ b/final_pricing.xlsx
@@ -713,12 +713,12 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>131000</t>
+          <t>131111</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Business Operations Specialists</t>
+          <t>Management Analysts</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -727,19 +727,19 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>46690</v>
+        <v>59720</v>
       </c>
       <c r="I7" t="n">
-        <v>60690</v>
+        <v>76770</v>
       </c>
       <c r="J7" t="n">
-        <v>80410</v>
+        <v>101190</v>
       </c>
       <c r="K7" t="n">
-        <v>108270</v>
+        <v>133140</v>
       </c>
       <c r="L7" t="n">
-        <v>143140</v>
+        <v>174140</v>
       </c>
     </row>
     <row r="8">
@@ -755,12 +755,12 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>131000</t>
+          <t>131111</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Business Operations Specialists</t>
+          <t>Management Analysts</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -769,19 +769,19 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>46690</v>
+        <v>59720</v>
       </c>
       <c r="I8" t="n">
-        <v>60690</v>
+        <v>76770</v>
       </c>
       <c r="J8" t="n">
-        <v>80410</v>
+        <v>101190</v>
       </c>
       <c r="K8" t="n">
-        <v>108270</v>
+        <v>133140</v>
       </c>
       <c r="L8" t="n">
-        <v>143140</v>
+        <v>174140</v>
       </c>
     </row>
     <row r="9">

</xml_diff>